<commit_message>
feat: Add Quarterly Backlog reporting with circle-wise generation
</commit_message>
<xml_diff>
--- a/src/components/Roster/filled.xlsx
+++ b/src/components/Roster/filled.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MYPRO\Roster\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MYPRO\pzhr_web\src\components\Roster\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DBA99B8-F01F-4C22-8F52-78A858D77FB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{272E051C-68DE-4738-963B-108C9B50E092}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{97B97223-865E-45D4-9E75-2997D7267C15}"/>
   </bookViews>
@@ -425,7 +425,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -581,6 +581,10 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -937,6 +941,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{52F914DD-9CA0-4F58-9507-29CB9EFA06D1}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:R59"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1004,7 +1009,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="2" spans="1:18" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:18" ht="20.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A2" s="35" t="s">
         <v>17</v>
       </c>
@@ -1055,7 +1060,7 @@
       </c>
       <c r="R2" s="8"/>
     </row>
-    <row r="3" spans="1:18" ht="20.25" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:18" ht="20.25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A3" s="35" t="s">
         <v>17</v>
       </c>
@@ -1106,7 +1111,7 @@
       </c>
       <c r="R3" s="8"/>
     </row>
-    <row r="4" spans="1:18" ht="20.25" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:18" ht="20.25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A4" s="35" t="s">
         <v>17</v>
       </c>
@@ -1157,7 +1162,7 @@
       </c>
       <c r="R4" s="6"/>
     </row>
-    <row r="5" spans="1:18" ht="20.25" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:18" ht="20.25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A5" s="35" t="s">
         <v>17</v>
       </c>
@@ -1208,7 +1213,7 @@
       </c>
       <c r="R5" s="6"/>
     </row>
-    <row r="6" spans="1:18" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:18" ht="20.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6" s="35" t="s">
         <v>17</v>
       </c>
@@ -1259,7 +1264,7 @@
       </c>
       <c r="R6" s="8"/>
     </row>
-    <row r="7" spans="1:18" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:18" ht="20.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A7" s="35" t="s">
         <v>17</v>
       </c>
@@ -1312,7 +1317,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="8" spans="1:18" ht="20.25" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:18" ht="20.25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A8" s="35" t="s">
         <v>17</v>
       </c>
@@ -1363,7 +1368,7 @@
       </c>
       <c r="R8" s="8"/>
     </row>
-    <row r="9" spans="1:18" ht="20.25" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:18" ht="20.25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A9" s="35" t="s">
         <v>17</v>
       </c>
@@ -1414,7 +1419,7 @@
       </c>
       <c r="R9" s="8"/>
     </row>
-    <row r="10" spans="1:18" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:18" ht="20.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A10" s="35" t="s">
         <v>17</v>
       </c>
@@ -1465,7 +1470,7 @@
       </c>
       <c r="R10" s="8"/>
     </row>
-    <row r="11" spans="1:18" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:18" ht="20.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A11" s="35" t="s">
         <v>17</v>
       </c>
@@ -1518,7 +1523,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="12" spans="1:18" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:18" ht="20.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A12" s="35" t="s">
         <v>17</v>
       </c>
@@ -1569,7 +1574,7 @@
       </c>
       <c r="R12" s="8"/>
     </row>
-    <row r="13" spans="1:18" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:18" ht="20.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A13" s="35" t="s">
         <v>17</v>
       </c>
@@ -1620,7 +1625,7 @@
       </c>
       <c r="R13" s="8"/>
     </row>
-    <row r="14" spans="1:18" ht="20.25" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:18" ht="20.25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A14" s="35" t="s">
         <v>17</v>
       </c>
@@ -1671,7 +1676,7 @@
       </c>
       <c r="R14" s="6"/>
     </row>
-    <row r="15" spans="1:18" ht="20.25" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:18" ht="20.25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A15" s="35" t="s">
         <v>17</v>
       </c>
@@ -1722,7 +1727,7 @@
       </c>
       <c r="R15" s="6"/>
     </row>
-    <row r="16" spans="1:18" ht="20.25" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:18" ht="20.25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A16" s="35" t="s">
         <v>17</v>
       </c>
@@ -1773,7 +1778,7 @@
       </c>
       <c r="R16" s="6"/>
     </row>
-    <row r="17" spans="1:18" ht="20.25" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:18" ht="20.25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A17" s="35" t="s">
         <v>17</v>
       </c>
@@ -1824,7 +1829,7 @@
       </c>
       <c r="R17" s="6"/>
     </row>
-    <row r="18" spans="1:18" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:18" ht="20.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18" s="35" t="s">
         <v>17</v>
       </c>
@@ -1875,7 +1880,7 @@
       </c>
       <c r="R18" s="8"/>
     </row>
-    <row r="19" spans="1:18" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:18" ht="20.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A19" s="35" t="s">
         <v>17</v>
       </c>
@@ -1928,7 +1933,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="20" spans="1:18" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:18" ht="20.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A20" s="35" t="s">
         <v>17</v>
       </c>
@@ -2595,7 +2600,7 @@
       </c>
       <c r="R32" s="8"/>
     </row>
-    <row r="33" spans="1:18" ht="20.25" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:18" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A33" s="36" t="s">
         <v>29</v>
       </c>
@@ -2606,40 +2611,42 @@
       <c r="D33" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="E33" s="6">
-        <v>1</v>
-      </c>
-      <c r="F33" s="6">
-        <v>1</v>
-      </c>
-      <c r="G33" s="6">
-        <v>1</v>
-      </c>
-      <c r="H33" s="6">
-        <v>0</v>
-      </c>
-      <c r="I33" s="6">
-        <v>0</v>
-      </c>
-      <c r="J33" s="6">
-        <v>0</v>
-      </c>
-      <c r="K33" s="6">
-        <v>0</v>
-      </c>
-      <c r="L33" s="6">
-        <v>0</v>
-      </c>
-      <c r="M33" s="6">
-        <v>0</v>
-      </c>
-      <c r="N33" s="6">
-        <v>0</v>
-      </c>
-      <c r="O33" s="6">
-        <v>16</v>
-      </c>
-      <c r="P33" s="6"/>
+      <c r="E33" s="5">
+        <v>1</v>
+      </c>
+      <c r="F33" s="5">
+        <v>1</v>
+      </c>
+      <c r="G33" s="5">
+        <v>1</v>
+      </c>
+      <c r="H33" s="5">
+        <v>0</v>
+      </c>
+      <c r="I33" s="5">
+        <v>0</v>
+      </c>
+      <c r="J33" s="5">
+        <v>0</v>
+      </c>
+      <c r="K33" s="5">
+        <v>0</v>
+      </c>
+      <c r="L33" s="5">
+        <v>0</v>
+      </c>
+      <c r="M33" s="5">
+        <v>0</v>
+      </c>
+      <c r="N33" s="5">
+        <v>0</v>
+      </c>
+      <c r="O33" s="5">
+        <v>15</v>
+      </c>
+      <c r="P33" s="3">
+        <v>1</v>
+      </c>
       <c r="Q33" s="3">
         <f t="shared" si="0"/>
         <v>19</v>
@@ -2657,40 +2664,42 @@
       <c r="D34" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="E34" s="6">
+      <c r="E34" s="5">
         <v>6</v>
       </c>
-      <c r="F34" s="6">
-        <v>2</v>
-      </c>
-      <c r="G34" s="6">
-        <v>2</v>
-      </c>
-      <c r="H34" s="6">
-        <v>0</v>
-      </c>
-      <c r="I34" s="6">
-        <v>3</v>
-      </c>
-      <c r="J34" s="6">
-        <v>1</v>
-      </c>
-      <c r="K34" s="6">
-        <v>0</v>
-      </c>
-      <c r="L34" s="6">
-        <v>0</v>
-      </c>
-      <c r="M34" s="6">
-        <v>0</v>
-      </c>
-      <c r="N34" s="6">
-        <v>0</v>
-      </c>
-      <c r="O34" s="6">
-        <v>103</v>
-      </c>
-      <c r="P34" s="6"/>
+      <c r="F34" s="5">
+        <v>2</v>
+      </c>
+      <c r="G34" s="5">
+        <v>1</v>
+      </c>
+      <c r="H34" s="5">
+        <v>0</v>
+      </c>
+      <c r="I34" s="5">
+        <v>2</v>
+      </c>
+      <c r="J34" s="5">
+        <v>1</v>
+      </c>
+      <c r="K34" s="5">
+        <v>0</v>
+      </c>
+      <c r="L34" s="5">
+        <v>0</v>
+      </c>
+      <c r="M34" s="5">
+        <v>0</v>
+      </c>
+      <c r="N34" s="5">
+        <v>0</v>
+      </c>
+      <c r="O34" s="5">
+        <v>101</v>
+      </c>
+      <c r="P34" s="6">
+        <v>4</v>
+      </c>
       <c r="Q34" s="3">
         <f t="shared" si="0"/>
         <v>117</v>
@@ -2838,7 +2847,7 @@
         <v>0</v>
       </c>
       <c r="N37" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O37" s="5">
         <v>80</v>
@@ -2846,7 +2855,7 @@
       <c r="P37" s="5"/>
       <c r="Q37" s="3">
         <f t="shared" si="0"/>
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="R37" s="8"/>
     </row>
@@ -2865,10 +2874,10 @@
         <v>0</v>
       </c>
       <c r="F38" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G38" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H38" s="5">
         <v>0</v>
@@ -2883,7 +2892,7 @@
         <v>0</v>
       </c>
       <c r="L38" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M38" s="5">
         <v>0</v>
@@ -2892,12 +2901,12 @@
         <v>1</v>
       </c>
       <c r="O38" s="5">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="P38" s="5"/>
       <c r="Q38" s="3">
         <f t="shared" si="0"/>
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="R38" s="8" t="s">
         <v>58</v>
@@ -2954,7 +2963,7 @@
       </c>
       <c r="R39" s="8"/>
     </row>
-    <row r="40" spans="1:18" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:18" ht="20.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A40" s="37" t="s">
         <v>30</v>
       </c>
@@ -3005,7 +3014,7 @@
       </c>
       <c r="R40" s="43"/>
     </row>
-    <row r="41" spans="1:18" ht="20.25" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:18" ht="20.25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A41" s="37" t="s">
         <v>30</v>
       </c>
@@ -3056,7 +3065,7 @@
       </c>
       <c r="R41" s="43"/>
     </row>
-    <row r="42" spans="1:18" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:18" ht="20.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A42" s="37" t="s">
         <v>30</v>
       </c>
@@ -3107,7 +3116,7 @@
       </c>
       <c r="R42" s="43"/>
     </row>
-    <row r="43" spans="1:18" ht="20.25" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:18" ht="20.25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A43" s="37" t="s">
         <v>30</v>
       </c>
@@ -3158,7 +3167,7 @@
       </c>
       <c r="R43" s="43"/>
     </row>
-    <row r="44" spans="1:18" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:18" ht="20.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A44" s="37" t="s">
         <v>30</v>
       </c>
@@ -3209,7 +3218,7 @@
       </c>
       <c r="R44" s="43"/>
     </row>
-    <row r="45" spans="1:18" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:18" ht="20.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A45" s="37" t="s">
         <v>30</v>
       </c>
@@ -3262,7 +3271,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="46" spans="1:18" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:18" ht="20.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A46" s="37" t="s">
         <v>30</v>
       </c>
@@ -3313,7 +3322,7 @@
       </c>
       <c r="R46" s="43"/>
     </row>
-    <row r="47" spans="1:18" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:18" ht="20.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A47" s="37" t="s">
         <v>30</v>
       </c>
@@ -3364,7 +3373,7 @@
       </c>
       <c r="R47" s="43"/>
     </row>
-    <row r="48" spans="1:18" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:18" ht="20.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A48" s="37" t="s">
         <v>30</v>
       </c>
@@ -3415,7 +3424,7 @@
       </c>
       <c r="R48" s="43"/>
     </row>
-    <row r="49" spans="1:18" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:18" ht="20.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A49" s="37" t="s">
         <v>30</v>
       </c>
@@ -3468,7 +3477,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="50" spans="1:18" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:18" ht="20.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A50" s="37" t="s">
         <v>30</v>
       </c>
@@ -3521,7 +3530,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="51" spans="1:18" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:18" ht="20.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A51" s="37" t="s">
         <v>30</v>
       </c>
@@ -3572,7 +3581,7 @@
       </c>
       <c r="R51" s="43"/>
     </row>
-    <row r="52" spans="1:18" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:18" ht="20.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A52" s="37" t="s">
         <v>30</v>
       </c>
@@ -3623,7 +3632,7 @@
       </c>
       <c r="R52" s="43"/>
     </row>
-    <row r="53" spans="1:18" ht="20.25" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:18" ht="20.25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A53" s="37" t="s">
         <v>30</v>
       </c>
@@ -3676,7 +3685,7 @@
       </c>
       <c r="R53" s="43"/>
     </row>
-    <row r="54" spans="1:18" ht="20.25" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:18" ht="20.25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A54" s="37" t="s">
         <v>30</v>
       </c>
@@ -3727,7 +3736,7 @@
       </c>
       <c r="R54" s="43"/>
     </row>
-    <row r="55" spans="1:18" ht="20.25" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:18" ht="20.25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A55" s="37" t="s">
         <v>30</v>
       </c>
@@ -3778,7 +3787,7 @@
       </c>
       <c r="R55" s="43"/>
     </row>
-    <row r="56" spans="1:18" ht="20.25" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:18" ht="20.25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A56" s="37" t="s">
         <v>30</v>
       </c>
@@ -3829,7 +3838,7 @@
       </c>
       <c r="R56" s="43"/>
     </row>
-    <row r="57" spans="1:18" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:18" ht="20.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A57" s="37" t="s">
         <v>30</v>
       </c>
@@ -3880,7 +3889,7 @@
       </c>
       <c r="R57" s="43"/>
     </row>
-    <row r="58" spans="1:18" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:18" ht="20.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A58" s="37" t="s">
         <v>30</v>
       </c>
@@ -3933,7 +3942,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="59" spans="1:18" ht="20.25" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:18" ht="20.25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A59" s="37" t="s">
         <v>30</v>
       </c>
@@ -3987,7 +3996,13 @@
       <c r="R59" s="43"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:R59" xr:uid="{52F914DD-9CA0-4F58-9507-29CB9EFA06D1}"/>
+  <autoFilter ref="A1:R59" xr:uid="{52F914DD-9CA0-4F58-9507-29CB9EFA06D1}">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="GKUC"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
@@ -3995,6 +4010,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AAF36A4E-756E-480F-94E4-598988175605}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:R85"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -4060,7 +4076,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="2" spans="1:18" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:18" ht="20.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>17</v>
       </c>
@@ -4113,7 +4129,7 @@
       </c>
       <c r="R2" s="8"/>
     </row>
-    <row r="3" spans="1:18" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:18" ht="20.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>17</v>
       </c>
@@ -4168,7 +4184,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="4" spans="1:18" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:18" ht="20.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>17</v>
       </c>
@@ -4221,7 +4237,7 @@
       </c>
       <c r="R4" s="8"/>
     </row>
-    <row r="5" spans="1:18" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:18" ht="20.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>17</v>
       </c>
@@ -4276,7 +4292,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="6" spans="1:18" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:18" ht="20.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>17</v>
       </c>
@@ -4329,7 +4345,7 @@
       </c>
       <c r="R6" s="8"/>
     </row>
-    <row r="7" spans="1:18" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:18" ht="20.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>17</v>
       </c>
@@ -4384,7 +4400,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="8" spans="1:18" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:18" ht="20.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>17</v>
       </c>
@@ -4437,7 +4453,7 @@
       </c>
       <c r="R8" s="8"/>
     </row>
-    <row r="9" spans="1:18" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:18" ht="20.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>17</v>
       </c>
@@ -4492,7 +4508,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="10" spans="1:18" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:18" ht="20.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>17</v>
       </c>
@@ -4545,7 +4561,7 @@
       </c>
       <c r="R10" s="8"/>
     </row>
-    <row r="11" spans="1:18" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:18" ht="18.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>17</v>
       </c>
@@ -5032,7 +5048,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="20" spans="1:18" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:18" ht="20.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>30</v>
       </c>
@@ -5085,7 +5101,7 @@
       </c>
       <c r="R20" s="8"/>
     </row>
-    <row r="21" spans="1:18" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:18" ht="20.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>30</v>
       </c>
@@ -5140,7 +5156,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="22" spans="1:18" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:18" ht="20.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>30</v>
       </c>
@@ -5193,7 +5209,7 @@
       </c>
       <c r="R22" s="8"/>
     </row>
-    <row r="23" spans="1:18" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:18" ht="20.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>30</v>
       </c>
@@ -5248,7 +5264,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="24" spans="1:18" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:18" ht="20.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>30</v>
       </c>
@@ -5301,7 +5317,7 @@
       </c>
       <c r="R24" s="8"/>
     </row>
-    <row r="25" spans="1:18" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:18" ht="20.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>30</v>
       </c>
@@ -5356,7 +5372,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="26" spans="1:18" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:18" ht="18.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
         <v>17</v>
       </c>
@@ -5409,7 +5425,7 @@
       </c>
       <c r="R26" s="8"/>
     </row>
-    <row r="27" spans="1:18" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:18" ht="18.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
         <v>17</v>
       </c>
@@ -5466,7 +5482,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="28" spans="1:18" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:18" ht="18.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>17</v>
       </c>
@@ -5519,7 +5535,7 @@
       </c>
       <c r="R28" s="8"/>
     </row>
-    <row r="29" spans="1:18" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:18" ht="18.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
         <v>17</v>
       </c>
@@ -5574,7 +5590,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="30" spans="1:18" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:18" ht="18.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>17</v>
       </c>
@@ -5627,7 +5643,7 @@
       </c>
       <c r="R30" s="8"/>
     </row>
-    <row r="31" spans="1:18" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:18" ht="18.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
         <v>17</v>
       </c>
@@ -5682,7 +5698,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="32" spans="1:18" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:18" ht="18.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>17</v>
       </c>
@@ -5735,7 +5751,7 @@
       </c>
       <c r="R32" s="8"/>
     </row>
-    <row r="33" spans="1:18" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:18" ht="18.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>17</v>
       </c>
@@ -5790,7 +5806,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="34" spans="1:18" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:18" ht="18.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
         <v>17</v>
       </c>
@@ -5843,7 +5859,7 @@
       </c>
       <c r="R34" s="8"/>
     </row>
-    <row r="35" spans="1:18" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:18" ht="18.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
         <v>17</v>
       </c>
@@ -6330,7 +6346,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="44" spans="1:18" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:18" ht="18.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
         <v>30</v>
       </c>
@@ -6383,7 +6399,7 @@
       </c>
       <c r="R44" s="8"/>
     </row>
-    <row r="45" spans="1:18" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:18" ht="18.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
         <v>30</v>
       </c>
@@ -6438,7 +6454,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="46" spans="1:18" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:18" ht="18.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
         <v>30</v>
       </c>
@@ -6491,7 +6507,7 @@
       </c>
       <c r="R46" s="8"/>
     </row>
-    <row r="47" spans="1:18" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:18" ht="20.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
         <v>30</v>
       </c>
@@ -6546,7 +6562,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="48" spans="1:18" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:18" ht="18.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
         <v>30</v>
       </c>
@@ -6599,7 +6615,7 @@
       </c>
       <c r="R48" s="8"/>
     </row>
-    <row r="49" spans="1:18" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:18" ht="20.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
         <v>30</v>
       </c>
@@ -6654,7 +6670,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="50" spans="1:18" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:18" ht="18.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
         <v>17</v>
       </c>
@@ -6707,7 +6723,7 @@
       </c>
       <c r="R50" s="8"/>
     </row>
-    <row r="51" spans="1:18" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:18" ht="18.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A51" s="2" t="s">
         <v>17</v>
       </c>
@@ -6760,7 +6776,7 @@
       </c>
       <c r="R51" s="8"/>
     </row>
-    <row r="52" spans="1:18" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:18" ht="18.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
         <v>17</v>
       </c>
@@ -6813,7 +6829,7 @@
       </c>
       <c r="R52" s="8"/>
     </row>
-    <row r="53" spans="1:18" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:18" ht="18.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A53" s="2" t="s">
         <v>17</v>
       </c>
@@ -6866,7 +6882,7 @@
       </c>
       <c r="R53" s="8"/>
     </row>
-    <row r="54" spans="1:18" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:18" ht="18.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A54" s="2" t="s">
         <v>17</v>
       </c>
@@ -7131,7 +7147,7 @@
       </c>
       <c r="R58" s="8"/>
     </row>
-    <row r="59" spans="1:18" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:18" ht="18.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A59" s="2" t="s">
         <v>30</v>
       </c>
@@ -7144,37 +7160,37 @@
       <c r="D59" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="E59" s="22">
-        <v>2</v>
-      </c>
-      <c r="F59" s="22">
-        <v>2</v>
-      </c>
-      <c r="G59" s="22">
-        <v>0</v>
-      </c>
-      <c r="H59" s="22">
-        <v>0</v>
-      </c>
-      <c r="I59" s="22">
-        <v>0</v>
-      </c>
-      <c r="J59" s="22">
-        <v>0</v>
-      </c>
-      <c r="K59" s="22">
-        <v>1</v>
-      </c>
-      <c r="L59" s="22">
-        <v>0</v>
-      </c>
-      <c r="M59" s="22">
-        <v>0</v>
-      </c>
-      <c r="N59" s="22">
-        <v>0</v>
-      </c>
-      <c r="O59" s="22">
+      <c r="E59" s="48">
+        <v>2</v>
+      </c>
+      <c r="F59" s="48">
+        <v>2</v>
+      </c>
+      <c r="G59" s="48">
+        <v>0</v>
+      </c>
+      <c r="H59" s="48">
+        <v>0</v>
+      </c>
+      <c r="I59" s="48">
+        <v>0</v>
+      </c>
+      <c r="J59" s="48">
+        <v>0</v>
+      </c>
+      <c r="K59" s="48">
+        <v>1</v>
+      </c>
+      <c r="L59" s="48">
+        <v>0</v>
+      </c>
+      <c r="M59" s="48">
+        <v>0</v>
+      </c>
+      <c r="N59" s="48">
+        <v>0</v>
+      </c>
+      <c r="O59" s="48">
         <v>103</v>
       </c>
       <c r="P59" s="22"/>
@@ -7184,7 +7200,7 @@
       </c>
       <c r="R59" s="8"/>
     </row>
-    <row r="60" spans="1:18" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:18" ht="18.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A60" s="2" t="s">
         <v>30</v>
       </c>
@@ -7237,7 +7253,7 @@
       </c>
       <c r="R60" s="8"/>
     </row>
-    <row r="61" spans="1:18" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:18" ht="20.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A61" s="2" t="s">
         <v>30</v>
       </c>
@@ -7250,37 +7266,37 @@
       <c r="D61" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="E61" s="11">
+      <c r="E61" s="5">
         <v>7</v>
       </c>
-      <c r="F61" s="11">
-        <v>1</v>
-      </c>
-      <c r="G61" s="11">
-        <v>1</v>
-      </c>
-      <c r="H61" s="11">
-        <v>1</v>
-      </c>
-      <c r="I61" s="11">
-        <v>1</v>
-      </c>
-      <c r="J61" s="11">
-        <v>2</v>
-      </c>
-      <c r="K61" s="11">
+      <c r="F61" s="5">
+        <v>1</v>
+      </c>
+      <c r="G61" s="5">
+        <v>1</v>
+      </c>
+      <c r="H61" s="5">
+        <v>1</v>
+      </c>
+      <c r="I61" s="5">
+        <v>1</v>
+      </c>
+      <c r="J61" s="5">
+        <v>2</v>
+      </c>
+      <c r="K61" s="5">
         <v>3</v>
       </c>
-      <c r="L61" s="11">
-        <v>0</v>
-      </c>
-      <c r="M61" s="11">
-        <v>0</v>
-      </c>
-      <c r="N61" s="11">
-        <v>0</v>
-      </c>
-      <c r="O61" s="11">
+      <c r="L61" s="5">
+        <v>0</v>
+      </c>
+      <c r="M61" s="5">
+        <v>0</v>
+      </c>
+      <c r="N61" s="5">
+        <v>0</v>
+      </c>
+      <c r="O61" s="5">
         <v>106</v>
       </c>
       <c r="P61" s="11"/>
@@ -7290,7 +7306,7 @@
       </c>
       <c r="R61" s="8"/>
     </row>
-    <row r="62" spans="1:18" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:18" ht="18.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A62" s="2" t="s">
         <v>17</v>
       </c>
@@ -7343,7 +7359,7 @@
       </c>
       <c r="R62" s="8"/>
     </row>
-    <row r="63" spans="1:18" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:18" ht="18.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A63" s="2" t="s">
         <v>17</v>
       </c>
@@ -7398,7 +7414,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="64" spans="1:18" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:18" ht="18.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A64" s="2" t="s">
         <v>17</v>
       </c>
@@ -7451,7 +7467,7 @@
       </c>
       <c r="R64" s="8"/>
     </row>
-    <row r="65" spans="1:18" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:18" ht="18.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A65" s="2" t="s">
         <v>17</v>
       </c>
@@ -7506,7 +7522,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="66" spans="1:18" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:18" ht="18.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A66" s="2" t="s">
         <v>17</v>
       </c>
@@ -7559,7 +7575,7 @@
       </c>
       <c r="R66" s="8"/>
     </row>
-    <row r="67" spans="1:18" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:18" ht="18.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A67" s="2" t="s">
         <v>17</v>
       </c>
@@ -7614,7 +7630,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="68" spans="1:18" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:18" ht="18.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A68" s="2" t="s">
         <v>17</v>
       </c>
@@ -7667,7 +7683,7 @@
       </c>
       <c r="R68" s="8"/>
     </row>
-    <row r="69" spans="1:18" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:18" ht="18.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A69" s="2" t="s">
         <v>17</v>
       </c>
@@ -7722,7 +7738,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="70" spans="1:18" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:18" ht="18.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A70" s="2" t="s">
         <v>17</v>
       </c>
@@ -7775,7 +7791,7 @@
       </c>
       <c r="R70" s="8"/>
     </row>
-    <row r="71" spans="1:18" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:18" ht="18.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A71" s="2" t="s">
         <v>17</v>
       </c>
@@ -8262,7 +8278,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="80" spans="1:18" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:18" ht="18.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A80" s="2" t="s">
         <v>30</v>
       </c>
@@ -8315,7 +8331,7 @@
       </c>
       <c r="R80" s="8"/>
     </row>
-    <row r="81" spans="1:18" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:18" ht="18.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A81" s="2" t="s">
         <v>30</v>
       </c>
@@ -8370,7 +8386,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="82" spans="1:18" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:18" ht="20.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A82" s="2" t="s">
         <v>30</v>
       </c>
@@ -8423,7 +8439,7 @@
       </c>
       <c r="R82" s="8"/>
     </row>
-    <row r="83" spans="1:18" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:18" ht="20.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A83" s="2" t="s">
         <v>30</v>
       </c>
@@ -8478,7 +8494,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="84" spans="1:18" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:18" ht="20.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A84" s="2" t="s">
         <v>30</v>
       </c>
@@ -8531,7 +8547,7 @@
       </c>
       <c r="R84" s="8"/>
     </row>
-    <row r="85" spans="1:18" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:18" ht="20.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A85" s="2" t="s">
         <v>30</v>
       </c>
@@ -8587,7 +8603,13 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:R85" xr:uid="{AAF36A4E-756E-480F-94E4-598988175605}"/>
+  <autoFilter ref="A1:R85" xr:uid="{AAF36A4E-756E-480F-94E4-598988175605}">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="GKUC"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>